<commit_message>
[Add - Weapon Data] 무기 데이터 추가 ( 검 / 창 )
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Weapon.xlsx
+++ b/JsonConverter/ExcelFiles/Weapon.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12458"/>
+  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12581"/>
   <x:workbookPr date1904="0" showBorderUnselectedTables="1" filterPrivacy="0" promptedSolutions="0" showInkAnnotation="1" backupFile="0" saveExternalLinkValues="1" codeName="ThisWorkbook" hidePivotFieldList="0" allowRefreshQuery="0" publishItems="0" checkCompatibility="0" autoCompressPictures="1" refreshAllConnections="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" Requires="x15">
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6720"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="18828" windowHeight="6792"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Weapon" sheetId="1" r:id="rId4"/>
@@ -19,24 +19,69 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 장창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>창술 수련에 사용되는 훈련용 창.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>설명</x:t>
+  </x:si>
   <x:si>
     <x:t>int</x:t>
   </x:si>
   <x:si>
-    <x:t>이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>커피</x:t>
+    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
   </x:si>
   <x:si>
     <x:t>웰빙리아 기사검</x:t>
@@ -48,43 +93,64 @@
     <x:t>Description</x:t>
   </x:si>
   <x:si>
-    <x:t>일순간 잉여가 될 수 있는 마법의 커피. 시공간을 분리시킨다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_Braclet_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_CoffeeCup_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>마법팔찌</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 왕국의 기사단이 사용하는 특별한 검.</x:t>
-  </x:si>
-  <x:si>
     <x:t>Icon/Icon_Weapon_Sword_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_Sword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>마법을 사용할 수 있는 팔찌</x:t>
-  </x:si>
-  <x:si>
-    <x:t>설명</x:t>
+    <x:t>Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토 장창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 기사검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 왕국 기사단이 사용하는 장창.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 힘을 이끌어내는 전용 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 왕국의 기사단에 지급되는 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 검술 훈련에 사용되는 표준 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSpear_1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -926,10 +992,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:P35"/>
+  <x:dimension ref="A1:P38"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
-    <x:col min="1" max="1" width="23" style="1" customWidth="1"/>
+    <x:col min="1" max="1" width="24.33203125" style="1" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="1" customWidth="1"/>
     <x:col min="3" max="3" width="52.5546875" style="1" customWidth="1"/>
     <x:col min="4" max="4" width="12.66796875" style="17" customWidth="1"/>
@@ -939,21 +1005,21 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A1" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>1</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D1" s="18" t="s">
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
         <x:v>14</x:v>
@@ -962,7 +1028,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="D2" s="18" t="s">
-        <x:v>0</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E2" s="14" t="s">
         <x:v>14</x:v>
@@ -970,36 +1036,36 @@
     </x:row>
     <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A3" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D3" s="19" t="s">
-        <x:v>3</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E3" s="15" t="s">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:16" ht="15.75" customHeight="1">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:16" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A4" s="5" t="s">
-        <x:v>19</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
       <x:c r="D4" s="20">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E4" s="16" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F4" s="4"/>
       <x:c r="G4" s="4"/>
@@ -1013,18 +1079,22 @@
       <x:c r="O4" s="4"/>
       <x:c r="P4" s="4"/>
     </x:row>
-    <x:row r="5" spans="1:16" ht="15.75" customHeight="1">
+    <x:row r="5" spans="1:16" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D5" s="20">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="D5" s="21"/>
-      <x:c r="E5" s="16"/>
+      <x:c r="E5" s="16" t="s">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F5" s="4"/>
       <x:c r="G5" s="4"/>
       <x:c r="H5" s="4"/>
@@ -1038,17 +1108,21 @@
       <x:c r="P5" s="4"/>
     </x:row>
     <x:row r="6" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A6" s="6" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="D6" s="21"/>
-      <x:c r="E6" s="16"/>
+      <x:c r="A6" s="5" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D6" s="20">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="F6" s="4"/>
       <x:c r="G6" s="4"/>
       <x:c r="H6" s="4"/>
@@ -1061,12 +1135,22 @@
       <x:c r="O6" s="4"/>
       <x:c r="P6" s="4"/>
     </x:row>
-    <x:row r="7" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A7" s="5"/>
-      <x:c r="B7" s="5"/>
-      <x:c r="C7" s="5"/>
-      <x:c r="D7" s="20"/>
-      <x:c r="E7" s="16"/>
+    <x:row r="7" spans="1:16" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A7" s="5" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D7" s="20">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="s">
+        <x:v>33</x:v>
+      </x:c>
       <x:c r="F7" s="4"/>
       <x:c r="G7" s="4"/>
       <x:c r="H7" s="4"/>
@@ -1080,11 +1164,21 @@
       <x:c r="P7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7"/>
-      <x:c r="C8" s="7"/>
-      <x:c r="D8" s="22"/>
-      <x:c r="E8" s="16"/>
+      <x:c r="A8" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="D8" s="21">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E8" s="16" t="s">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="F8" s="4"/>
       <x:c r="G8" s="4"/>
       <x:c r="H8" s="4"/>
@@ -1098,11 +1192,21 @@
       <x:c r="P8" s="4"/>
     </x:row>
     <x:row r="9" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A9" s="7"/>
-      <x:c r="B9" s="7"/>
-      <x:c r="C9" s="7"/>
-      <x:c r="D9" s="22"/>
-      <x:c r="E9" s="16"/>
+      <x:c r="A9" s="6" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D9" s="21">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E9" s="16" t="s">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="F9" s="4"/>
       <x:c r="G9" s="4"/>
       <x:c r="H9" s="4"/>
@@ -1116,11 +1220,21 @@
       <x:c r="P9" s="4"/>
     </x:row>
     <x:row r="10" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A10" s="8"/>
-      <x:c r="B10" s="8"/>
-      <x:c r="C10" s="8"/>
-      <x:c r="D10" s="23"/>
-      <x:c r="E10" s="16"/>
+      <x:c r="A10" s="5" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D10" s="20">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E10" s="16" t="s">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="F10" s="4"/>
       <x:c r="G10" s="4"/>
       <x:c r="H10" s="4"/>
@@ -1134,11 +1248,21 @@
       <x:c r="P10" s="4"/>
     </x:row>
     <x:row r="11" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A11" s="8"/>
-      <x:c r="B11" s="8"/>
-      <x:c r="C11" s="8"/>
-      <x:c r="D11" s="23"/>
-      <x:c r="E11" s="16"/>
+      <x:c r="A11" s="7" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D11" s="22">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E11" s="16" t="s">
+        <x:v>27</x:v>
+      </x:c>
       <x:c r="F11" s="4"/>
       <x:c r="G11" s="4"/>
       <x:c r="H11" s="4"/>
@@ -1170,10 +1294,10 @@
       <x:c r="P12" s="4"/>
     </x:row>
     <x:row r="13" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A13" s="5"/>
-      <x:c r="B13" s="5"/>
-      <x:c r="C13" s="5"/>
-      <x:c r="D13" s="20"/>
+      <x:c r="A13" s="8"/>
+      <x:c r="B13" s="8"/>
+      <x:c r="C13" s="8"/>
+      <x:c r="D13" s="23"/>
       <x:c r="E13" s="16"/>
       <x:c r="F13" s="4"/>
       <x:c r="G13" s="4"/>
@@ -1206,10 +1330,10 @@
       <x:c r="P14" s="4"/>
     </x:row>
     <x:row r="15" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A15" s="8"/>
-      <x:c r="B15" s="8"/>
-      <x:c r="C15" s="8"/>
-      <x:c r="D15" s="23"/>
+      <x:c r="A15" s="7"/>
+      <x:c r="B15" s="7"/>
+      <x:c r="C15" s="7"/>
+      <x:c r="D15" s="22"/>
       <x:c r="E15" s="16"/>
       <x:c r="F15" s="4"/>
       <x:c r="G15" s="4"/>
@@ -1223,30 +1347,65 @@
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
     </x:row>
-    <x:row r="16" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A16" s="9"/>
-      <x:c r="B16" s="9"/>
-      <x:c r="C16" s="9"/>
-      <x:c r="D16" s="24"/>
-    </x:row>
-    <x:row r="17" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A17" s="10"/>
-      <x:c r="B17" s="10"/>
-      <x:c r="C17" s="10"/>
-      <x:c r="D17" s="24"/>
-    </x:row>
-    <x:row r="18" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A18" s="10"/>
-      <x:c r="B18" s="10"/>
-      <x:c r="C18" s="10"/>
-      <x:c r="D18" s="24"/>
-    </x:row>
-    <x:row r="19" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A19" s="10"/>
-      <x:c r="B19" s="10"/>
-      <x:c r="C19" s="10"/>
+    <x:row r="16" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A16" s="5"/>
+      <x:c r="B16" s="5"/>
+      <x:c r="C16" s="5"/>
+      <x:c r="D16" s="20"/>
+      <x:c r="E16" s="16"/>
+      <x:c r="F16" s="4"/>
+      <x:c r="G16" s="4"/>
+      <x:c r="H16" s="4"/>
+      <x:c r="I16" s="4"/>
+      <x:c r="J16" s="4"/>
+      <x:c r="K16" s="4"/>
+      <x:c r="L16" s="4"/>
+      <x:c r="M16" s="4"/>
+      <x:c r="N16" s="4"/>
+      <x:c r="O16" s="4"/>
+      <x:c r="P16" s="4"/>
+    </x:row>
+    <x:row r="17" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A17" s="8"/>
+      <x:c r="B17" s="8"/>
+      <x:c r="C17" s="8"/>
+      <x:c r="D17" s="23"/>
+      <x:c r="E17" s="16"/>
+      <x:c r="F17" s="4"/>
+      <x:c r="G17" s="4"/>
+      <x:c r="H17" s="4"/>
+      <x:c r="I17" s="4"/>
+      <x:c r="J17" s="4"/>
+      <x:c r="K17" s="4"/>
+      <x:c r="L17" s="4"/>
+      <x:c r="M17" s="4"/>
+      <x:c r="N17" s="4"/>
+      <x:c r="O17" s="4"/>
+      <x:c r="P17" s="4"/>
+    </x:row>
+    <x:row r="18" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A18" s="8"/>
+      <x:c r="B18" s="8"/>
+      <x:c r="C18" s="8"/>
+      <x:c r="D18" s="23"/>
+      <x:c r="E18" s="16"/>
+      <x:c r="F18" s="4"/>
+      <x:c r="G18" s="4"/>
+      <x:c r="H18" s="4"/>
+      <x:c r="I18" s="4"/>
+      <x:c r="J18" s="4"/>
+      <x:c r="K18" s="4"/>
+      <x:c r="L18" s="4"/>
+      <x:c r="M18" s="4"/>
+      <x:c r="N18" s="4"/>
+      <x:c r="O18" s="4"/>
+      <x:c r="P18" s="4"/>
+    </x:row>
+    <x:row r="19" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A19" s="9"/>
+      <x:c r="B19" s="9"/>
+      <x:c r="C19" s="9"/>
       <x:c r="D19" s="24"/>
-      <x:c r="F19" s="4"/>
     </x:row>
     <x:row r="20" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A20" s="10"/>
@@ -1260,11 +1419,12 @@
       <x:c r="C21" s="10"/>
       <x:c r="D21" s="24"/>
     </x:row>
-    <x:row r="22" spans="1:4" ht="15.75" customHeight="1">
+    <x:row r="22" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A22" s="10"/>
       <x:c r="B22" s="10"/>
       <x:c r="C22" s="10"/>
       <x:c r="D22" s="24"/>
+      <x:c r="F22" s="4"/>
     </x:row>
     <x:row r="23" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A23" s="10"/>
@@ -1278,69 +1438,69 @@
       <x:c r="C24" s="10"/>
       <x:c r="D24" s="24"/>
     </x:row>
-    <x:row r="25" spans="1:6" ht="15.75" customHeight="1">
+    <x:row r="25" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A25" s="10"/>
       <x:c r="B25" s="10"/>
       <x:c r="C25" s="10"/>
       <x:c r="D25" s="24"/>
-      <x:c r="F25" s="4"/>
-    </x:row>
-    <x:row r="26" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A26" s="11"/>
-      <x:c r="B26" s="11"/>
-      <x:c r="C26" s="11"/>
-      <x:c r="D26" s="25"/>
-      <x:c r="F26" s="4"/>
-    </x:row>
-    <x:row r="27" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A27" s="11"/>
-      <x:c r="B27" s="11"/>
-      <x:c r="C27" s="11"/>
-      <x:c r="D27" s="25"/>
-      <x:c r="F27" s="4"/>
+    </x:row>
+    <x:row r="26" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A26" s="10"/>
+      <x:c r="B26" s="10"/>
+      <x:c r="C26" s="10"/>
+      <x:c r="D26" s="24"/>
+    </x:row>
+    <x:row r="27" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A27" s="10"/>
+      <x:c r="B27" s="10"/>
+      <x:c r="C27" s="10"/>
+      <x:c r="D27" s="24"/>
     </x:row>
     <x:row r="28" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A28" s="11"/>
-      <x:c r="B28" s="11"/>
-      <x:c r="C28" s="11"/>
-      <x:c r="D28" s="25"/>
+      <x:c r="A28" s="10"/>
+      <x:c r="B28" s="10"/>
+      <x:c r="C28" s="10"/>
+      <x:c r="D28" s="24"/>
       <x:c r="F28" s="4"/>
     </x:row>
-    <x:row r="29" spans="1:4" ht="15.75" customHeight="1">
+    <x:row r="29" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A29" s="11"/>
       <x:c r="B29" s="11"/>
       <x:c r="C29" s="11"/>
       <x:c r="D29" s="25"/>
-    </x:row>
-    <x:row r="30" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="F29" s="4"/>
+    </x:row>
+    <x:row r="30" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A30" s="11"/>
       <x:c r="B30" s="11"/>
       <x:c r="C30" s="11"/>
       <x:c r="D30" s="25"/>
-    </x:row>
-    <x:row r="31" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="F30" s="4"/>
+    </x:row>
+    <x:row r="31" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A31" s="11"/>
       <x:c r="B31" s="11"/>
       <x:c r="C31" s="11"/>
       <x:c r="D31" s="25"/>
+      <x:c r="F31" s="4"/>
     </x:row>
     <x:row r="32" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A32" s="12"/>
-      <x:c r="B32" s="12"/>
-      <x:c r="C32" s="12"/>
-      <x:c r="D32" s="26"/>
+      <x:c r="A32" s="11"/>
+      <x:c r="B32" s="11"/>
+      <x:c r="C32" s="11"/>
+      <x:c r="D32" s="25"/>
     </x:row>
     <x:row r="33" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A33" s="12"/>
-      <x:c r="B33" s="12"/>
-      <x:c r="C33" s="12"/>
-      <x:c r="D33" s="26"/>
+      <x:c r="A33" s="11"/>
+      <x:c r="B33" s="11"/>
+      <x:c r="C33" s="11"/>
+      <x:c r="D33" s="25"/>
     </x:row>
     <x:row r="34" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A34" s="12"/>
-      <x:c r="B34" s="12"/>
-      <x:c r="C34" s="12"/>
-      <x:c r="D34" s="26"/>
+      <x:c r="A34" s="11"/>
+      <x:c r="B34" s="11"/>
+      <x:c r="C34" s="11"/>
+      <x:c r="D34" s="25"/>
     </x:row>
     <x:row r="35" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A35" s="12"/>
@@ -1348,9 +1508,24 @@
       <x:c r="C35" s="12"/>
       <x:c r="D35" s="26"/>
     </x:row>
-    <x:row r="36" ht="15.75" customHeight="1"/>
-    <x:row r="37" ht="15.75" customHeight="1"/>
-    <x:row r="38" ht="15.75" customHeight="1"/>
+    <x:row r="36" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A36" s="12"/>
+      <x:c r="B36" s="12"/>
+      <x:c r="C36" s="12"/>
+      <x:c r="D36" s="26"/>
+    </x:row>
+    <x:row r="37" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A37" s="12"/>
+      <x:c r="B37" s="12"/>
+      <x:c r="C37" s="12"/>
+      <x:c r="D37" s="26"/>
+    </x:row>
+    <x:row r="38" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="A38" s="12"/>
+      <x:c r="B38" s="12"/>
+      <x:c r="C38" s="12"/>
+      <x:c r="D38" s="26"/>
+    </x:row>
     <x:row r="39" ht="15.75" customHeight="1"/>
     <x:row r="40" ht="15.75" customHeight="1"/>
     <x:row r="41" ht="15.75" customHeight="1"/>
@@ -2313,6 +2488,9 @@
     <x:row r="998" ht="15.75" customHeight="1"/>
     <x:row r="999" ht="15.75" customHeight="1"/>
     <x:row r="1000" ht="15.75" customHeight="1"/>
+    <x:row r="1001" ht="15.75" customHeight="1"/>
+    <x:row r="1002" ht="15.75" customHeight="1"/>
+    <x:row r="1003" ht="15.75" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="0" fitToHeight="0" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>

<commit_message>
[Fix - Weapon Data] 웰빙리아 기사검 IconPath 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Weapon.xlsx
+++ b/JsonConverter/ExcelFiles/Weapon.xlsx
@@ -21,136 +21,136 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <x:si>
+    <x:t>창술 수련에 사용되는 훈련용 창.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 힘을 이끌어내는 전용 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
   </x:si>
   <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>설명</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 기사검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토 장창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
     <x:t>웰빙리아 장창</x:t>
   </x:si>
   <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 기사검</x:t>
+  </x:si>
+  <x:si>
     <x:t>나무 검</x:t>
   </x:si>
   <x:si>
-    <x:t>나무 창</x:t>
+    <x:t>웰빙리아 왕국 기사단이 사용하는 장창.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 왕국의 기사단에 지급되는 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 검술 훈련에 사용되는 표준 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSword_1</x:t>
   </x:si>
   <x:si>
     <x:t>Weapon_WellbeingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WellbeingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>훈련용 검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>창술 수련에 사용되는 훈련용 창.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>설명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_Sword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TrainingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토 장창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토의 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 왕국 기사단이 사용하는 장창.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토의 힘을 이끌어내는 전용 검.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>훈련용 창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WoodenSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 왕국의 기사단에 지급되는 검.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 검술 훈련에 사용되는 표준 검.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TrainingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TotoSpear_1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -306,7 +306,10 @@
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="28">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:alignment horizontal="general" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
@@ -995,536 +998,536 @@
   <x:dimension ref="A1:P38"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
-    <x:col min="1" max="1" width="24.33203125" style="1" customWidth="1"/>
-    <x:col min="2" max="2" width="19.5703125" style="1" customWidth="1"/>
-    <x:col min="3" max="3" width="52.5546875" style="1" customWidth="1"/>
-    <x:col min="4" max="4" width="12.66796875" style="17" customWidth="1"/>
-    <x:col min="5" max="5" width="43.109375" style="13" customWidth="1"/>
-    <x:col min="6" max="6" width="30.5703125" style="1" customWidth="1"/>
+    <x:col min="1" max="1" width="24.33203125" style="2" customWidth="1"/>
+    <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="52.5546875" style="2" customWidth="1"/>
+    <x:col min="4" max="4" width="12.66796875" style="18" customWidth="1"/>
+    <x:col min="5" max="5" width="43.109375" style="14" customWidth="1"/>
+    <x:col min="6" max="6" width="30.5703125" style="2" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A1" s="2" t="s">
+      <x:c r="A1" s="3" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D1" s="19" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="A2" s="3" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C2" s="3" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="D2" s="19" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E2" s="15" t="s">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="A3" s="4" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A4" s="6" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D4" s="21">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F4" s="5"/>
+      <x:c r="G4" s="5"/>
+      <x:c r="H4" s="5"/>
+      <x:c r="I4" s="5"/>
+      <x:c r="J4" s="5"/>
+      <x:c r="K4" s="5"/>
+      <x:c r="L4" s="5"/>
+      <x:c r="M4" s="5"/>
+      <x:c r="N4" s="5"/>
+      <x:c r="O4" s="5"/>
+      <x:c r="P4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A5" s="6" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D5" s="21">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
+      <x:c r="F5" s="5"/>
+      <x:c r="G5" s="5"/>
+      <x:c r="H5" s="5"/>
+      <x:c r="I5" s="5"/>
+      <x:c r="J5" s="5"/>
+      <x:c r="K5" s="5"/>
+      <x:c r="L5" s="5"/>
+      <x:c r="M5" s="5"/>
+      <x:c r="N5" s="5"/>
+      <x:c r="O5" s="5"/>
+      <x:c r="P5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A6" s="6" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D6" s="21">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F6" s="5"/>
+      <x:c r="G6" s="5"/>
+      <x:c r="H6" s="5"/>
+      <x:c r="I6" s="5"/>
+      <x:c r="J6" s="5"/>
+      <x:c r="K6" s="5"/>
+      <x:c r="L6" s="5"/>
+      <x:c r="M6" s="5"/>
+      <x:c r="N6" s="5"/>
+      <x:c r="O6" s="5"/>
+      <x:c r="P6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A7" s="6" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D7" s="21">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F7" s="5"/>
+      <x:c r="G7" s="5"/>
+      <x:c r="H7" s="5"/>
+      <x:c r="I7" s="5"/>
+      <x:c r="J7" s="5"/>
+      <x:c r="K7" s="5"/>
+      <x:c r="L7" s="5"/>
+      <x:c r="M7" s="5"/>
+      <x:c r="N7" s="5"/>
+      <x:c r="O7" s="5"/>
+      <x:c r="P7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A8" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D8" s="22">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F8" s="5"/>
+      <x:c r="G8" s="5"/>
+      <x:c r="H8" s="5"/>
+      <x:c r="I8" s="5"/>
+      <x:c r="J8" s="5"/>
+      <x:c r="K8" s="5"/>
+      <x:c r="L8" s="5"/>
+      <x:c r="M8" s="5"/>
+      <x:c r="N8" s="5"/>
+      <x:c r="O8" s="5"/>
+      <x:c r="P8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A9" s="7" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="22">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="D1" s="18" t="s">
+      <x:c r="E9" s="17" t="s">
         <x:v>11</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A2" s="2" t="s">
+      <x:c r="F9" s="5"/>
+      <x:c r="G9" s="5"/>
+      <x:c r="H9" s="5"/>
+      <x:c r="I9" s="5"/>
+      <x:c r="J9" s="5"/>
+      <x:c r="K9" s="5"/>
+      <x:c r="L9" s="5"/>
+      <x:c r="M9" s="5"/>
+      <x:c r="N9" s="5"/>
+      <x:c r="O9" s="5"/>
+      <x:c r="P9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A10" s="6" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D10" s="21">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C2" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D2" s="18" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E2" s="14" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A3" s="3" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="s">
+      <x:c r="F10" s="5"/>
+      <x:c r="G10" s="5"/>
+      <x:c r="H10" s="5"/>
+      <x:c r="I10" s="5"/>
+      <x:c r="J10" s="5"/>
+      <x:c r="K10" s="5"/>
+      <x:c r="L10" s="5"/>
+      <x:c r="M10" s="5"/>
+      <x:c r="N10" s="5"/>
+      <x:c r="O10" s="5"/>
+      <x:c r="P10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="A11" s="8" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="D3" s="19" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E3" s="15" t="s">
-        <x:v>22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:16" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A4" s="5" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D4" s="20">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F4" s="4"/>
-      <x:c r="G4" s="4"/>
-      <x:c r="H4" s="4"/>
-      <x:c r="I4" s="4"/>
-      <x:c r="J4" s="4"/>
-      <x:c r="K4" s="4"/>
-      <x:c r="L4" s="4"/>
-      <x:c r="M4" s="4"/>
-      <x:c r="N4" s="4"/>
-      <x:c r="O4" s="4"/>
-      <x:c r="P4" s="4"/>
-    </x:row>
-    <x:row r="5" spans="1:16" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A5" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B5" s="5" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="D5" s="20">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E5" s="16" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="4"/>
-      <x:c r="G5" s="4"/>
-      <x:c r="H5" s="4"/>
-      <x:c r="I5" s="4"/>
-      <x:c r="J5" s="4"/>
-      <x:c r="K5" s="4"/>
-      <x:c r="L5" s="4"/>
-      <x:c r="M5" s="4"/>
-      <x:c r="N5" s="4"/>
-      <x:c r="O5" s="4"/>
-      <x:c r="P5" s="4"/>
-    </x:row>
-    <x:row r="6" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A6" s="5" t="s">
+      <x:c r="C11" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="D6" s="20">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E6" s="16" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F6" s="4"/>
-      <x:c r="G6" s="4"/>
-      <x:c r="H6" s="4"/>
-      <x:c r="I6" s="4"/>
-      <x:c r="J6" s="4"/>
-      <x:c r="K6" s="4"/>
-      <x:c r="L6" s="4"/>
-      <x:c r="M6" s="4"/>
-      <x:c r="N6" s="4"/>
-      <x:c r="O6" s="4"/>
-      <x:c r="P6" s="4"/>
-    </x:row>
-    <x:row r="7" spans="1:16" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A7" s="5" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="D7" s="20">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E7" s="16" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="F7" s="4"/>
-      <x:c r="G7" s="4"/>
-      <x:c r="H7" s="4"/>
-      <x:c r="I7" s="4"/>
-      <x:c r="J7" s="4"/>
-      <x:c r="K7" s="4"/>
-      <x:c r="L7" s="4"/>
-      <x:c r="M7" s="4"/>
-      <x:c r="N7" s="4"/>
-      <x:c r="O7" s="4"/>
-      <x:c r="P7" s="4"/>
-    </x:row>
-    <x:row r="8" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A8" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="D8" s="21">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E8" s="16" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F8" s="4"/>
-      <x:c r="G8" s="4"/>
-      <x:c r="H8" s="4"/>
-      <x:c r="I8" s="4"/>
-      <x:c r="J8" s="4"/>
-      <x:c r="K8" s="4"/>
-      <x:c r="L8" s="4"/>
-      <x:c r="M8" s="4"/>
-      <x:c r="N8" s="4"/>
-      <x:c r="O8" s="4"/>
-      <x:c r="P8" s="4"/>
-    </x:row>
-    <x:row r="9" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A9" s="6" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D9" s="21">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E9" s="16" t="s">
+      <x:c r="D11" s="23">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="F9" s="4"/>
-      <x:c r="G9" s="4"/>
-      <x:c r="H9" s="4"/>
-      <x:c r="I9" s="4"/>
-      <x:c r="J9" s="4"/>
-      <x:c r="K9" s="4"/>
-      <x:c r="L9" s="4"/>
-      <x:c r="M9" s="4"/>
-      <x:c r="N9" s="4"/>
-      <x:c r="O9" s="4"/>
-      <x:c r="P9" s="4"/>
-    </x:row>
-    <x:row r="10" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A10" s="5" t="s">
+      <x:c r="E11" s="17" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D10" s="20">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E10" s="16" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F10" s="4"/>
-      <x:c r="G10" s="4"/>
-      <x:c r="H10" s="4"/>
-      <x:c r="I10" s="4"/>
-      <x:c r="J10" s="4"/>
-      <x:c r="K10" s="4"/>
-      <x:c r="L10" s="4"/>
-      <x:c r="M10" s="4"/>
-      <x:c r="N10" s="4"/>
-      <x:c r="O10" s="4"/>
-      <x:c r="P10" s="4"/>
-    </x:row>
-    <x:row r="11" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A11" s="7" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="D11" s="22">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E11" s="16" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="F11" s="4"/>
-      <x:c r="G11" s="4"/>
-      <x:c r="H11" s="4"/>
-      <x:c r="I11" s="4"/>
-      <x:c r="J11" s="4"/>
-      <x:c r="K11" s="4"/>
-      <x:c r="L11" s="4"/>
-      <x:c r="M11" s="4"/>
-      <x:c r="N11" s="4"/>
-      <x:c r="O11" s="4"/>
-      <x:c r="P11" s="4"/>
+      <x:c r="F11" s="5"/>
+      <x:c r="G11" s="5"/>
+      <x:c r="H11" s="5"/>
+      <x:c r="I11" s="5"/>
+      <x:c r="J11" s="5"/>
+      <x:c r="K11" s="5"/>
+      <x:c r="L11" s="5"/>
+      <x:c r="M11" s="5"/>
+      <x:c r="N11" s="5"/>
+      <x:c r="O11" s="5"/>
+      <x:c r="P11" s="5"/>
     </x:row>
     <x:row r="12" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A12" s="7"/>
-      <x:c r="B12" s="7"/>
-      <x:c r="C12" s="7"/>
-      <x:c r="D12" s="22"/>
-      <x:c r="E12" s="16"/>
-      <x:c r="F12" s="4"/>
-      <x:c r="G12" s="4"/>
-      <x:c r="H12" s="4"/>
-      <x:c r="I12" s="4"/>
-      <x:c r="J12" s="4"/>
-      <x:c r="K12" s="4"/>
-      <x:c r="L12" s="4"/>
-      <x:c r="M12" s="4"/>
-      <x:c r="N12" s="4"/>
-      <x:c r="O12" s="4"/>
-      <x:c r="P12" s="4"/>
+      <x:c r="A12" s="8"/>
+      <x:c r="B12" s="8"/>
+      <x:c r="C12" s="8"/>
+      <x:c r="D12" s="23"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="5"/>
+      <x:c r="G12" s="5"/>
+      <x:c r="H12" s="5"/>
+      <x:c r="I12" s="5"/>
+      <x:c r="J12" s="5"/>
+      <x:c r="K12" s="5"/>
+      <x:c r="L12" s="5"/>
+      <x:c r="M12" s="5"/>
+      <x:c r="N12" s="5"/>
+      <x:c r="O12" s="5"/>
+      <x:c r="P12" s="5"/>
     </x:row>
     <x:row r="13" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A13" s="8"/>
-      <x:c r="B13" s="8"/>
-      <x:c r="C13" s="8"/>
-      <x:c r="D13" s="23"/>
-      <x:c r="E13" s="16"/>
-      <x:c r="F13" s="4"/>
-      <x:c r="G13" s="4"/>
-      <x:c r="H13" s="4"/>
-      <x:c r="I13" s="4"/>
-      <x:c r="J13" s="4"/>
-      <x:c r="K13" s="4"/>
-      <x:c r="L13" s="4"/>
-      <x:c r="M13" s="4"/>
-      <x:c r="N13" s="4"/>
-      <x:c r="O13" s="4"/>
-      <x:c r="P13" s="4"/>
+      <x:c r="A13" s="9"/>
+      <x:c r="B13" s="9"/>
+      <x:c r="C13" s="9"/>
+      <x:c r="D13" s="24"/>
+      <x:c r="E13" s="17"/>
+      <x:c r="F13" s="5"/>
+      <x:c r="G13" s="5"/>
+      <x:c r="H13" s="5"/>
+      <x:c r="I13" s="5"/>
+      <x:c r="J13" s="5"/>
+      <x:c r="K13" s="5"/>
+      <x:c r="L13" s="5"/>
+      <x:c r="M13" s="5"/>
+      <x:c r="N13" s="5"/>
+      <x:c r="O13" s="5"/>
+      <x:c r="P13" s="5"/>
     </x:row>
     <x:row r="14" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A14" s="8"/>
-      <x:c r="B14" s="8"/>
-      <x:c r="C14" s="8"/>
-      <x:c r="D14" s="23"/>
-      <x:c r="E14" s="16"/>
-      <x:c r="F14" s="4"/>
-      <x:c r="G14" s="4"/>
-      <x:c r="H14" s="4"/>
-      <x:c r="I14" s="4"/>
-      <x:c r="J14" s="4"/>
-      <x:c r="K14" s="4"/>
-      <x:c r="L14" s="4"/>
-      <x:c r="M14" s="4"/>
-      <x:c r="N14" s="4"/>
-      <x:c r="O14" s="4"/>
-      <x:c r="P14" s="4"/>
+      <x:c r="A14" s="9"/>
+      <x:c r="B14" s="9"/>
+      <x:c r="C14" s="9"/>
+      <x:c r="D14" s="24"/>
+      <x:c r="E14" s="17"/>
+      <x:c r="F14" s="5"/>
+      <x:c r="G14" s="5"/>
+      <x:c r="H14" s="5"/>
+      <x:c r="I14" s="5"/>
+      <x:c r="J14" s="5"/>
+      <x:c r="K14" s="5"/>
+      <x:c r="L14" s="5"/>
+      <x:c r="M14" s="5"/>
+      <x:c r="N14" s="5"/>
+      <x:c r="O14" s="5"/>
+      <x:c r="P14" s="5"/>
     </x:row>
     <x:row r="15" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A15" s="7"/>
-      <x:c r="B15" s="7"/>
-      <x:c r="C15" s="7"/>
-      <x:c r="D15" s="22"/>
-      <x:c r="E15" s="16"/>
-      <x:c r="F15" s="4"/>
-      <x:c r="G15" s="4"/>
-      <x:c r="H15" s="4"/>
-      <x:c r="I15" s="4"/>
-      <x:c r="J15" s="4"/>
-      <x:c r="K15" s="4"/>
-      <x:c r="L15" s="4"/>
-      <x:c r="M15" s="4"/>
-      <x:c r="N15" s="4"/>
-      <x:c r="O15" s="4"/>
-      <x:c r="P15" s="4"/>
+      <x:c r="A15" s="8"/>
+      <x:c r="B15" s="8"/>
+      <x:c r="C15" s="8"/>
+      <x:c r="D15" s="23"/>
+      <x:c r="E15" s="17"/>
+      <x:c r="F15" s="5"/>
+      <x:c r="G15" s="5"/>
+      <x:c r="H15" s="5"/>
+      <x:c r="I15" s="5"/>
+      <x:c r="J15" s="5"/>
+      <x:c r="K15" s="5"/>
+      <x:c r="L15" s="5"/>
+      <x:c r="M15" s="5"/>
+      <x:c r="N15" s="5"/>
+      <x:c r="O15" s="5"/>
+      <x:c r="P15" s="5"/>
     </x:row>
     <x:row r="16" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A16" s="5"/>
-      <x:c r="B16" s="5"/>
-      <x:c r="C16" s="5"/>
-      <x:c r="D16" s="20"/>
-      <x:c r="E16" s="16"/>
-      <x:c r="F16" s="4"/>
-      <x:c r="G16" s="4"/>
-      <x:c r="H16" s="4"/>
-      <x:c r="I16" s="4"/>
-      <x:c r="J16" s="4"/>
-      <x:c r="K16" s="4"/>
-      <x:c r="L16" s="4"/>
-      <x:c r="M16" s="4"/>
-      <x:c r="N16" s="4"/>
-      <x:c r="O16" s="4"/>
-      <x:c r="P16" s="4"/>
+      <x:c r="A16" s="6"/>
+      <x:c r="B16" s="6"/>
+      <x:c r="C16" s="6"/>
+      <x:c r="D16" s="21"/>
+      <x:c r="E16" s="17"/>
+      <x:c r="F16" s="5"/>
+      <x:c r="G16" s="5"/>
+      <x:c r="H16" s="5"/>
+      <x:c r="I16" s="5"/>
+      <x:c r="J16" s="5"/>
+      <x:c r="K16" s="5"/>
+      <x:c r="L16" s="5"/>
+      <x:c r="M16" s="5"/>
+      <x:c r="N16" s="5"/>
+      <x:c r="O16" s="5"/>
+      <x:c r="P16" s="5"/>
     </x:row>
     <x:row r="17" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A17" s="8"/>
-      <x:c r="B17" s="8"/>
-      <x:c r="C17" s="8"/>
-      <x:c r="D17" s="23"/>
-      <x:c r="E17" s="16"/>
-      <x:c r="F17" s="4"/>
-      <x:c r="G17" s="4"/>
-      <x:c r="H17" s="4"/>
-      <x:c r="I17" s="4"/>
-      <x:c r="J17" s="4"/>
-      <x:c r="K17" s="4"/>
-      <x:c r="L17" s="4"/>
-      <x:c r="M17" s="4"/>
-      <x:c r="N17" s="4"/>
-      <x:c r="O17" s="4"/>
-      <x:c r="P17" s="4"/>
+      <x:c r="A17" s="9"/>
+      <x:c r="B17" s="9"/>
+      <x:c r="C17" s="9"/>
+      <x:c r="D17" s="24"/>
+      <x:c r="E17" s="17"/>
+      <x:c r="F17" s="5"/>
+      <x:c r="G17" s="5"/>
+      <x:c r="H17" s="5"/>
+      <x:c r="I17" s="5"/>
+      <x:c r="J17" s="5"/>
+      <x:c r="K17" s="5"/>
+      <x:c r="L17" s="5"/>
+      <x:c r="M17" s="5"/>
+      <x:c r="N17" s="5"/>
+      <x:c r="O17" s="5"/>
+      <x:c r="P17" s="5"/>
     </x:row>
     <x:row r="18" spans="1:16" ht="15.75" customHeight="1">
-      <x:c r="A18" s="8"/>
-      <x:c r="B18" s="8"/>
-      <x:c r="C18" s="8"/>
-      <x:c r="D18" s="23"/>
-      <x:c r="E18" s="16"/>
-      <x:c r="F18" s="4"/>
-      <x:c r="G18" s="4"/>
-      <x:c r="H18" s="4"/>
-      <x:c r="I18" s="4"/>
-      <x:c r="J18" s="4"/>
-      <x:c r="K18" s="4"/>
-      <x:c r="L18" s="4"/>
-      <x:c r="M18" s="4"/>
-      <x:c r="N18" s="4"/>
-      <x:c r="O18" s="4"/>
-      <x:c r="P18" s="4"/>
+      <x:c r="A18" s="9"/>
+      <x:c r="B18" s="9"/>
+      <x:c r="C18" s="9"/>
+      <x:c r="D18" s="24"/>
+      <x:c r="E18" s="17"/>
+      <x:c r="F18" s="5"/>
+      <x:c r="G18" s="5"/>
+      <x:c r="H18" s="5"/>
+      <x:c r="I18" s="5"/>
+      <x:c r="J18" s="5"/>
+      <x:c r="K18" s="5"/>
+      <x:c r="L18" s="5"/>
+      <x:c r="M18" s="5"/>
+      <x:c r="N18" s="5"/>
+      <x:c r="O18" s="5"/>
+      <x:c r="P18" s="5"/>
     </x:row>
     <x:row r="19" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A19" s="9"/>
-      <x:c r="B19" s="9"/>
-      <x:c r="C19" s="9"/>
-      <x:c r="D19" s="24"/>
+      <x:c r="A19" s="10"/>
+      <x:c r="B19" s="10"/>
+      <x:c r="C19" s="10"/>
+      <x:c r="D19" s="25"/>
     </x:row>
     <x:row r="20" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A20" s="10"/>
-      <x:c r="B20" s="10"/>
-      <x:c r="C20" s="10"/>
-      <x:c r="D20" s="24"/>
+      <x:c r="A20" s="11"/>
+      <x:c r="B20" s="11"/>
+      <x:c r="C20" s="11"/>
+      <x:c r="D20" s="25"/>
     </x:row>
     <x:row r="21" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A21" s="10"/>
-      <x:c r="B21" s="10"/>
-      <x:c r="C21" s="10"/>
-      <x:c r="D21" s="24"/>
+      <x:c r="A21" s="11"/>
+      <x:c r="B21" s="11"/>
+      <x:c r="C21" s="11"/>
+      <x:c r="D21" s="25"/>
     </x:row>
     <x:row r="22" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A22" s="10"/>
-      <x:c r="B22" s="10"/>
-      <x:c r="C22" s="10"/>
-      <x:c r="D22" s="24"/>
-      <x:c r="F22" s="4"/>
+      <x:c r="A22" s="11"/>
+      <x:c r="B22" s="11"/>
+      <x:c r="C22" s="11"/>
+      <x:c r="D22" s="25"/>
+      <x:c r="F22" s="5"/>
     </x:row>
     <x:row r="23" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A23" s="10"/>
-      <x:c r="B23" s="10"/>
-      <x:c r="C23" s="10"/>
-      <x:c r="D23" s="24"/>
+      <x:c r="A23" s="11"/>
+      <x:c r="B23" s="11"/>
+      <x:c r="C23" s="11"/>
+      <x:c r="D23" s="25"/>
     </x:row>
     <x:row r="24" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A24" s="10"/>
-      <x:c r="B24" s="10"/>
-      <x:c r="C24" s="10"/>
-      <x:c r="D24" s="24"/>
+      <x:c r="A24" s="11"/>
+      <x:c r="B24" s="11"/>
+      <x:c r="C24" s="11"/>
+      <x:c r="D24" s="25"/>
     </x:row>
     <x:row r="25" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A25" s="10"/>
-      <x:c r="B25" s="10"/>
-      <x:c r="C25" s="10"/>
-      <x:c r="D25" s="24"/>
+      <x:c r="A25" s="11"/>
+      <x:c r="B25" s="11"/>
+      <x:c r="C25" s="11"/>
+      <x:c r="D25" s="25"/>
     </x:row>
     <x:row r="26" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A26" s="10"/>
-      <x:c r="B26" s="10"/>
-      <x:c r="C26" s="10"/>
-      <x:c r="D26" s="24"/>
+      <x:c r="A26" s="11"/>
+      <x:c r="B26" s="11"/>
+      <x:c r="C26" s="11"/>
+      <x:c r="D26" s="25"/>
     </x:row>
     <x:row r="27" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A27" s="10"/>
-      <x:c r="B27" s="10"/>
-      <x:c r="C27" s="10"/>
-      <x:c r="D27" s="24"/>
+      <x:c r="A27" s="11"/>
+      <x:c r="B27" s="11"/>
+      <x:c r="C27" s="11"/>
+      <x:c r="D27" s="25"/>
     </x:row>
     <x:row r="28" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A28" s="10"/>
-      <x:c r="B28" s="10"/>
-      <x:c r="C28" s="10"/>
-      <x:c r="D28" s="24"/>
-      <x:c r="F28" s="4"/>
+      <x:c r="A28" s="11"/>
+      <x:c r="B28" s="11"/>
+      <x:c r="C28" s="11"/>
+      <x:c r="D28" s="25"/>
+      <x:c r="F28" s="5"/>
     </x:row>
     <x:row r="29" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A29" s="11"/>
-      <x:c r="B29" s="11"/>
-      <x:c r="C29" s="11"/>
-      <x:c r="D29" s="25"/>
-      <x:c r="F29" s="4"/>
+      <x:c r="A29" s="12"/>
+      <x:c r="B29" s="12"/>
+      <x:c r="C29" s="12"/>
+      <x:c r="D29" s="26"/>
+      <x:c r="F29" s="5"/>
     </x:row>
     <x:row r="30" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A30" s="11"/>
-      <x:c r="B30" s="11"/>
-      <x:c r="C30" s="11"/>
-      <x:c r="D30" s="25"/>
-      <x:c r="F30" s="4"/>
+      <x:c r="A30" s="12"/>
+      <x:c r="B30" s="12"/>
+      <x:c r="C30" s="12"/>
+      <x:c r="D30" s="26"/>
+      <x:c r="F30" s="5"/>
     </x:row>
     <x:row r="31" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A31" s="11"/>
-      <x:c r="B31" s="11"/>
-      <x:c r="C31" s="11"/>
-      <x:c r="D31" s="25"/>
-      <x:c r="F31" s="4"/>
+      <x:c r="A31" s="12"/>
+      <x:c r="B31" s="12"/>
+      <x:c r="C31" s="12"/>
+      <x:c r="D31" s="26"/>
+      <x:c r="F31" s="5"/>
     </x:row>
     <x:row r="32" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A32" s="11"/>
-      <x:c r="B32" s="11"/>
-      <x:c r="C32" s="11"/>
-      <x:c r="D32" s="25"/>
+      <x:c r="A32" s="12"/>
+      <x:c r="B32" s="12"/>
+      <x:c r="C32" s="12"/>
+      <x:c r="D32" s="26"/>
     </x:row>
     <x:row r="33" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A33" s="11"/>
-      <x:c r="B33" s="11"/>
-      <x:c r="C33" s="11"/>
-      <x:c r="D33" s="25"/>
+      <x:c r="A33" s="12"/>
+      <x:c r="B33" s="12"/>
+      <x:c r="C33" s="12"/>
+      <x:c r="D33" s="26"/>
     </x:row>
     <x:row r="34" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A34" s="11"/>
-      <x:c r="B34" s="11"/>
-      <x:c r="C34" s="11"/>
-      <x:c r="D34" s="25"/>
+      <x:c r="A34" s="12"/>
+      <x:c r="B34" s="12"/>
+      <x:c r="C34" s="12"/>
+      <x:c r="D34" s="26"/>
     </x:row>
     <x:row r="35" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A35" s="12"/>
-      <x:c r="B35" s="12"/>
-      <x:c r="C35" s="12"/>
-      <x:c r="D35" s="26"/>
+      <x:c r="A35" s="13"/>
+      <x:c r="B35" s="13"/>
+      <x:c r="C35" s="13"/>
+      <x:c r="D35" s="27"/>
     </x:row>
     <x:row r="36" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A36" s="12"/>
-      <x:c r="B36" s="12"/>
-      <x:c r="C36" s="12"/>
-      <x:c r="D36" s="26"/>
+      <x:c r="A36" s="13"/>
+      <x:c r="B36" s="13"/>
+      <x:c r="C36" s="13"/>
+      <x:c r="D36" s="27"/>
     </x:row>
     <x:row r="37" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A37" s="12"/>
-      <x:c r="B37" s="12"/>
-      <x:c r="C37" s="12"/>
-      <x:c r="D37" s="26"/>
+      <x:c r="A37" s="13"/>
+      <x:c r="B37" s="13"/>
+      <x:c r="C37" s="13"/>
+      <x:c r="D37" s="27"/>
     </x:row>
     <x:row r="38" spans="1:4" ht="15.75" customHeight="1">
-      <x:c r="A38" s="12"/>
-      <x:c r="B38" s="12"/>
-      <x:c r="C38" s="12"/>
-      <x:c r="D38" s="26"/>
+      <x:c r="A38" s="13"/>
+      <x:c r="B38" s="13"/>
+      <x:c r="C38" s="13"/>
+      <x:c r="D38" s="27"/>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1"/>
     <x:row r="40" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[Add - Weapon Data] RequiredLevel 데이터 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Weapon.xlsx
+++ b/JsonConverter/ExcelFiles/Weapon.xlsx
@@ -19,138 +19,144 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>설명</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 힘을 이끌어내는 전용 검.</x:t>
+  </x:si>
   <x:si>
     <x:t>창술 수련에 사용되는 훈련용 창.</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>Weapon_TotoSpear_1</x:t>
   </x:si>
   <x:si>
-    <x:t>토토의 힘을 이끌어내는 전용 검.</x:t>
+    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다.</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>설명</x:t>
-  </x:si>
-  <x:si>
     <x:t>Description</x:t>
   </x:si>
   <x:si>
+    <x:t>웰빙리아 기사검</x:t>
+  </x:si>
+  <x:si>
     <x:t>IconPath</x:t>
   </x:si>
   <x:si>
-    <x:t>웰빙리아 기사검</x:t>
+    <x:t>훈련용 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토 장창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 기사검</x:t>
   </x:si>
   <x:si>
     <x:t>훈련용 검</x:t>
   </x:si>
   <x:si>
-    <x:t>토토 장창</x:t>
+    <x:t>웰빙리아 장창</x:t>
   </x:si>
   <x:si>
     <x:t>Name</x:t>
   </x:si>
   <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>훈련용 창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무 창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 장창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토의 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무 검</x:t>
+    <x:t>웰빙리아 왕국의 기사단에 지급되는 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 검술 훈련에 사용되는 표준 검.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSpear_1</x:t>
   </x:si>
   <x:si>
     <x:t>웰빙리아 왕국 기사단이 사용하는 장창.</x:t>
   </x:si>
   <x:si>
-    <x:t>웰빙리아 왕국의 기사단에 지급되는 검.</x:t>
-  </x:si>
-  <x:si>
     <x:t>Weapon_WoodenSpear_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_TrainingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 검술 훈련에 사용되는 표준 검.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TrainingSword_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>Weapon_WellbeingSword_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_WellbeingSpear_1</x:t>
+    <x:t>요구 레벨</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiredLevel</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -199,7 +205,7 @@
       <x:color rgb="ff008000"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -242,8 +248,26 @@
         <x:bgColor indexed="64"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor indexed="65"/>
+        <x:bgColor rgb="ff000000"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="ffc6efce"/>
+        <x:bgColor rgb="ff000000"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="ffffffff"/>
+        <x:bgColor rgb="ff000000"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="5">
     <x:border>
       <x:left>
         <x:color auto="1"/>
@@ -273,7 +297,7 @@
       </x:bottom>
     </x:border>
     <x:border>
-      <x:left style="thin">
+      <x:left>
         <x:color auto="1"/>
       </x:left>
       <x:right style="thin">
@@ -294,10 +318,24 @@
         <x:color auto="1"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color auto="1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color auto="1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color auto="1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color auto="1"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -306,7 +344,7 @@
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
@@ -389,6 +427,21 @@
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
@@ -995,82 +1048,94 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:P38"/>
+  <x:dimension ref="A1:Q38"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="24.33203125" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="52.5546875" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="12.66796875" style="18" customWidth="1"/>
-    <x:col min="5" max="5" width="43.109375" style="14" customWidth="1"/>
-    <x:col min="6" max="6" width="30.5703125" style="2" customWidth="1"/>
+    <x:col min="5" max="5" width="14.77734375" style="28" customWidth="1"/>
+    <x:col min="6" max="6" width="43.109375" style="14" customWidth="1"/>
+    <x:col min="7" max="7" width="30.5703125" style="2" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:4" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B1" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C1" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D1" s="19" t="s">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5" ht="15.75" customHeight="1">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="s">
+        <x:v>44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>31</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>31</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D2" s="19" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E2" s="15" t="s">
-        <x:v>31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" ht="15.75" customHeight="1">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E2" s="29" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F2" s="15" t="s">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B3" s="4" t="s">
-        <x:v>24</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C3" s="4" t="s">
         <x:v>19</x:v>
       </x:c>
       <x:c r="D3" s="20" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="E3" s="16" t="s">
-        <x:v>20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E3" s="30" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A4" s="6" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B4" s="6" t="s">
-        <x:v>34</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C4" s="6" t="s">
-        <x:v>6</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D4" s="21">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E4" s="17" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F4" s="5"/>
+      <x:c r="E4" s="31">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F4" s="17" t="s">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5"/>
@@ -1081,24 +1146,27 @@
       <x:c r="N4" s="5"/>
       <x:c r="O4" s="5"/>
       <x:c r="P4" s="5"/>
-    </x:row>
-    <x:row r="5" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>41</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>22</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>39</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D5" s="21">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E5" s="17" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F5" s="5"/>
+      <x:c r="E5" s="31">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="s">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5"/>
@@ -1109,24 +1177,27 @@
       <x:c r="N5" s="5"/>
       <x:c r="O5" s="5"/>
       <x:c r="P5" s="5"/>
-    </x:row>
-    <x:row r="6" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C6" s="6" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D6" s="21">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="E6" s="17" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F6" s="5"/>
+      <x:c r="E6" s="31">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="s">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5"/>
@@ -1137,24 +1208,27 @@
       <x:c r="N6" s="5"/>
       <x:c r="O6" s="5"/>
       <x:c r="P6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="Q6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>1</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
-        <x:v>3</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="21">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="E7" s="17" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F7" s="5"/>
+      <x:c r="E7" s="31">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="s">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5"/>
@@ -1165,24 +1239,27 @@
       <x:c r="N7" s="5"/>
       <x:c r="O7" s="5"/>
       <x:c r="P7" s="5"/>
-    </x:row>
-    <x:row r="8" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A8" s="6" t="s">
-        <x:v>37</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D8" s="22">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E8" s="17" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F8" s="5"/>
+      <x:c r="E8" s="31">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="s">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5"/>
@@ -1193,24 +1270,27 @@
       <x:c r="N8" s="5"/>
       <x:c r="O8" s="5"/>
       <x:c r="P8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A9" s="7" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>26</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D9" s="22">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="E9" s="17" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="F9" s="5"/>
+      <x:c r="E9" s="31">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="s">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5"/>
@@ -1221,24 +1301,27 @@
       <x:c r="N9" s="5"/>
       <x:c r="O9" s="5"/>
       <x:c r="P9" s="5"/>
-    </x:row>
-    <x:row r="10" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A10" s="6" t="s">
-        <x:v>43</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B10" s="6" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C10" s="6" t="s">
-        <x:v>35</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D10" s="21">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="E10" s="17" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F10" s="5"/>
+      <x:c r="E10" s="31">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="s">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="G10" s="5"/>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5"/>
@@ -1249,24 +1332,27 @@
       <x:c r="N10" s="5"/>
       <x:c r="O10" s="5"/>
       <x:c r="P10" s="5"/>
-    </x:row>
-    <x:row r="11" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A11" s="8" t="s">
-        <x:v>2</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="8" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C11" s="8" t="s">
-        <x:v>7</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D11" s="23">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E11" s="17" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F11" s="5"/>
+      <x:c r="E11" s="31">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F11" s="17" t="s">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="G11" s="5"/>
       <x:c r="H11" s="5"/>
       <x:c r="I11" s="5"/>
@@ -1277,14 +1363,15 @@
       <x:c r="N11" s="5"/>
       <x:c r="O11" s="5"/>
       <x:c r="P11" s="5"/>
-    </x:row>
-    <x:row r="12" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A12" s="8"/>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="8"/>
       <x:c r="D12" s="23"/>
-      <x:c r="E12" s="17"/>
-      <x:c r="F12" s="5"/>
+      <x:c r="E12" s="31"/>
+      <x:c r="F12" s="17"/>
       <x:c r="G12" s="5"/>
       <x:c r="H12" s="5"/>
       <x:c r="I12" s="5"/>
@@ -1295,14 +1382,15 @@
       <x:c r="N12" s="5"/>
       <x:c r="O12" s="5"/>
       <x:c r="P12" s="5"/>
-    </x:row>
-    <x:row r="13" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q12" s="5"/>
+    </x:row>
+    <x:row r="13" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A13" s="9"/>
       <x:c r="B13" s="9"/>
       <x:c r="C13" s="9"/>
       <x:c r="D13" s="24"/>
-      <x:c r="E13" s="17"/>
-      <x:c r="F13" s="5"/>
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="17"/>
       <x:c r="G13" s="5"/>
       <x:c r="H13" s="5"/>
       <x:c r="I13" s="5"/>
@@ -1313,14 +1401,15 @@
       <x:c r="N13" s="5"/>
       <x:c r="O13" s="5"/>
       <x:c r="P13" s="5"/>
-    </x:row>
-    <x:row r="14" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q13" s="5"/>
+    </x:row>
+    <x:row r="14" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A14" s="9"/>
       <x:c r="B14" s="9"/>
       <x:c r="C14" s="9"/>
       <x:c r="D14" s="24"/>
-      <x:c r="E14" s="17"/>
-      <x:c r="F14" s="5"/>
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="17"/>
       <x:c r="G14" s="5"/>
       <x:c r="H14" s="5"/>
       <x:c r="I14" s="5"/>
@@ -1331,14 +1420,15 @@
       <x:c r="N14" s="5"/>
       <x:c r="O14" s="5"/>
       <x:c r="P14" s="5"/>
-    </x:row>
-    <x:row r="15" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q14" s="5"/>
+    </x:row>
+    <x:row r="15" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A15" s="8"/>
       <x:c r="B15" s="8"/>
       <x:c r="C15" s="8"/>
       <x:c r="D15" s="23"/>
-      <x:c r="E15" s="17"/>
-      <x:c r="F15" s="5"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="17"/>
       <x:c r="G15" s="5"/>
       <x:c r="H15" s="5"/>
       <x:c r="I15" s="5"/>
@@ -1349,14 +1439,15 @@
       <x:c r="N15" s="5"/>
       <x:c r="O15" s="5"/>
       <x:c r="P15" s="5"/>
-    </x:row>
-    <x:row r="16" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q15" s="5"/>
+    </x:row>
+    <x:row r="16" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A16" s="6"/>
       <x:c r="B16" s="6"/>
       <x:c r="C16" s="6"/>
       <x:c r="D16" s="21"/>
-      <x:c r="E16" s="17"/>
-      <x:c r="F16" s="5"/>
+      <x:c r="E16" s="31"/>
+      <x:c r="F16" s="17"/>
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="5"/>
       <x:c r="I16" s="5"/>
@@ -1367,14 +1458,15 @@
       <x:c r="N16" s="5"/>
       <x:c r="O16" s="5"/>
       <x:c r="P16" s="5"/>
-    </x:row>
-    <x:row r="17" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q16" s="5"/>
+    </x:row>
+    <x:row r="17" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A17" s="9"/>
       <x:c r="B17" s="9"/>
       <x:c r="C17" s="9"/>
       <x:c r="D17" s="24"/>
-      <x:c r="E17" s="17"/>
-      <x:c r="F17" s="5"/>
+      <x:c r="E17" s="31"/>
+      <x:c r="F17" s="17"/>
       <x:c r="G17" s="5"/>
       <x:c r="H17" s="5"/>
       <x:c r="I17" s="5"/>
@@ -1385,14 +1477,15 @@
       <x:c r="N17" s="5"/>
       <x:c r="O17" s="5"/>
       <x:c r="P17" s="5"/>
-    </x:row>
-    <x:row r="18" spans="1:16" ht="15.75" customHeight="1">
+      <x:c r="Q17" s="5"/>
+    </x:row>
+    <x:row r="18" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A18" s="9"/>
       <x:c r="B18" s="9"/>
       <x:c r="C18" s="9"/>
       <x:c r="D18" s="24"/>
-      <x:c r="E18" s="17"/>
-      <x:c r="F18" s="5"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="17"/>
       <x:c r="G18" s="5"/>
       <x:c r="H18" s="5"/>
       <x:c r="I18" s="5"/>
@@ -1403,131 +1496,152 @@
       <x:c r="N18" s="5"/>
       <x:c r="O18" s="5"/>
       <x:c r="P18" s="5"/>
-    </x:row>
-    <x:row r="19" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="Q18" s="5"/>
+    </x:row>
+    <x:row r="19" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A19" s="10"/>
       <x:c r="B19" s="10"/>
       <x:c r="C19" s="10"/>
       <x:c r="D19" s="25"/>
-    </x:row>
-    <x:row r="20" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E19" s="32"/>
+    </x:row>
+    <x:row r="20" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A20" s="11"/>
       <x:c r="B20" s="11"/>
       <x:c r="C20" s="11"/>
       <x:c r="D20" s="25"/>
-    </x:row>
-    <x:row r="21" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E20" s="32"/>
+    </x:row>
+    <x:row r="21" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A21" s="11"/>
       <x:c r="B21" s="11"/>
       <x:c r="C21" s="11"/>
       <x:c r="D21" s="25"/>
-    </x:row>
-    <x:row r="22" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E21" s="32"/>
+    </x:row>
+    <x:row r="22" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A22" s="11"/>
       <x:c r="B22" s="11"/>
       <x:c r="C22" s="11"/>
       <x:c r="D22" s="25"/>
-      <x:c r="F22" s="5"/>
-    </x:row>
-    <x:row r="23" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E22" s="32"/>
+      <x:c r="G22" s="5"/>
+    </x:row>
+    <x:row r="23" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A23" s="11"/>
       <x:c r="B23" s="11"/>
       <x:c r="C23" s="11"/>
       <x:c r="D23" s="25"/>
-    </x:row>
-    <x:row r="24" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E23" s="32"/>
+    </x:row>
+    <x:row r="24" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A24" s="11"/>
       <x:c r="B24" s="11"/>
       <x:c r="C24" s="11"/>
       <x:c r="D24" s="25"/>
-    </x:row>
-    <x:row r="25" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E24" s="32"/>
+    </x:row>
+    <x:row r="25" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A25" s="11"/>
       <x:c r="B25" s="11"/>
       <x:c r="C25" s="11"/>
       <x:c r="D25" s="25"/>
-    </x:row>
-    <x:row r="26" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E25" s="32"/>
+    </x:row>
+    <x:row r="26" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A26" s="11"/>
       <x:c r="B26" s="11"/>
       <x:c r="C26" s="11"/>
       <x:c r="D26" s="25"/>
-    </x:row>
-    <x:row r="27" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E26" s="32"/>
+    </x:row>
+    <x:row r="27" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A27" s="11"/>
       <x:c r="B27" s="11"/>
       <x:c r="C27" s="11"/>
       <x:c r="D27" s="25"/>
-    </x:row>
-    <x:row r="28" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E27" s="32"/>
+    </x:row>
+    <x:row r="28" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A28" s="11"/>
       <x:c r="B28" s="11"/>
       <x:c r="C28" s="11"/>
       <x:c r="D28" s="25"/>
-      <x:c r="F28" s="5"/>
-    </x:row>
-    <x:row r="29" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E28" s="32"/>
+      <x:c r="G28" s="5"/>
+    </x:row>
+    <x:row r="29" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A29" s="12"/>
       <x:c r="B29" s="12"/>
       <x:c r="C29" s="12"/>
       <x:c r="D29" s="26"/>
-      <x:c r="F29" s="5"/>
-    </x:row>
-    <x:row r="30" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E29" s="32"/>
+      <x:c r="G29" s="5"/>
+    </x:row>
+    <x:row r="30" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A30" s="12"/>
       <x:c r="B30" s="12"/>
       <x:c r="C30" s="12"/>
       <x:c r="D30" s="26"/>
-      <x:c r="F30" s="5"/>
-    </x:row>
-    <x:row r="31" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="E30" s="32"/>
+      <x:c r="G30" s="5"/>
+    </x:row>
+    <x:row r="31" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A31" s="12"/>
       <x:c r="B31" s="12"/>
       <x:c r="C31" s="12"/>
       <x:c r="D31" s="26"/>
-      <x:c r="F31" s="5"/>
-    </x:row>
-    <x:row r="32" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E31" s="32"/>
+      <x:c r="G31" s="5"/>
+    </x:row>
+    <x:row r="32" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A32" s="12"/>
       <x:c r="B32" s="12"/>
       <x:c r="C32" s="12"/>
       <x:c r="D32" s="26"/>
-    </x:row>
-    <x:row r="33" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E32" s="32"/>
+    </x:row>
+    <x:row r="33" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A33" s="12"/>
       <x:c r="B33" s="12"/>
       <x:c r="C33" s="12"/>
       <x:c r="D33" s="26"/>
-    </x:row>
-    <x:row r="34" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E33" s="32"/>
+    </x:row>
+    <x:row r="34" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A34" s="12"/>
       <x:c r="B34" s="12"/>
       <x:c r="C34" s="12"/>
       <x:c r="D34" s="26"/>
-    </x:row>
-    <x:row r="35" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E34" s="32"/>
+    </x:row>
+    <x:row r="35" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A35" s="13"/>
       <x:c r="B35" s="13"/>
       <x:c r="C35" s="13"/>
       <x:c r="D35" s="27"/>
-    </x:row>
-    <x:row r="36" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E35" s="32"/>
+    </x:row>
+    <x:row r="36" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A36" s="13"/>
       <x:c r="B36" s="13"/>
       <x:c r="C36" s="13"/>
       <x:c r="D36" s="27"/>
-    </x:row>
-    <x:row r="37" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E36" s="32"/>
+    </x:row>
+    <x:row r="37" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A37" s="13"/>
       <x:c r="B37" s="13"/>
       <x:c r="C37" s="13"/>
       <x:c r="D37" s="27"/>
-    </x:row>
-    <x:row r="38" spans="1:4" ht="15.75" customHeight="1">
+      <x:c r="E37" s="32"/>
+    </x:row>
+    <x:row r="38" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A38" s="13"/>
       <x:c r="B38" s="13"/>
       <x:c r="C38" s="13"/>
       <x:c r="D38" s="27"/>
+      <x:c r="E38" s="32"/>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1"/>
     <x:row r="40" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[Fix - Weapon Data] 설명에 공격력 기재
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Weapon.xlsx
+++ b/JsonConverter/ExcelFiles/Weapon.xlsx
@@ -21,142 +21,142 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
   <x:si>
+    <x:t>웰빙리아 왕국 기사단이 사용하는 장창. (공격력+ 24)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>창술 수련에 사용되는 훈련용 창. (공격력+ 18)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 힘을 이끌어내는 전용 검. (공격력+ 25)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 왕국의 기사단에 지급되는 검. (공격력+ 20)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다. (공격력+ 12)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다. (공격력+ 30)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>설명</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 검술 훈련에 사용되는 표준 검. (공격력+ 15)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 기사검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>설명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
+    <x:t>RequiredLevel</x:t>
   </x:si>
   <x:si>
     <x:t>Weapon_TotoSword_1</x:t>
   </x:si>
   <x:si>
-    <x:t>토토의 힘을 이끌어내는 전용 검.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>창술 수련에 사용되는 훈련용 창.</x:t>
-  </x:si>
-  <x:si>
     <x:t>Weapon_TotoSpear_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
   </x:si>
   <x:si>
     <x:t>훈련용 창</x:t>
   </x:si>
   <x:si>
+    <x:t>나무 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
     <x:t>나무 창</x:t>
   </x:si>
   <x:si>
+    <x:t>웰빙리아 장창</x:t>
+  </x:si>
+  <x:si>
     <x:t>토토 장창</x:t>
   </x:si>
   <x:si>
-    <x:t>나무 검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
+    <x:t>토토의 기사검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>요구 레벨</x:t>
   </x:si>
   <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
-    <x:t>토토의 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>훈련용 검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 장창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 왕국의 기사단에 지급되는 검.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 검술 훈련에 사용되는 표준 검.</x:t>
+    <x:t>Weapon_TrainingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSpear_1</x:t>
   </x:si>
   <x:si>
     <x:t>Weapon_TrainingSword_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_WellbeingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TrainingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 왕국 기사단이 사용하는 장창.</x:t>
+    <x:t>Weapon_WellbeingSword_1</x:t>
   </x:si>
   <x:si>
     <x:t>Weapon_WoodenSpear_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_WellbeingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>요구 레벨</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RequiredLevel</x:t>
+    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다. (공격력+ 10)</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1053,7 +1053,7 @@
   <x:cols>
     <x:col min="1" max="1" width="24.33203125" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
-    <x:col min="3" max="3" width="52.5546875" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="60.4453125" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="12.66796875" style="18" customWidth="1"/>
     <x:col min="5" max="5" width="14.77734375" style="28" customWidth="1"/>
     <x:col min="6" max="6" width="43.109375" style="14" customWidth="1"/>
@@ -1062,70 +1062,70 @@
   <x:sheetData>
     <x:row r="1" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D1" s="19" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D1" s="19" t="s">
-        <x:v>26</x:v>
-      </x:c>
       <x:c r="E1" s="29" t="s">
-        <x:v>44</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>30</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="19" t="s">
-        <x:v>4</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E2" s="29" t="s">
-        <x:v>4</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F2" s="15" t="s">
-        <x:v>27</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
-        <x:v>6</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B3" s="4" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C3" s="4" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D3" s="20" t="s">
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E3" s="30" t="s">
-        <x:v>45</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F3" s="16" t="s">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A4" s="6" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B4" s="6" t="s">
-        <x:v>25</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C4" s="6" t="s">
-        <x:v>13</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D4" s="21">
         <x:v>10</x:v>
@@ -1134,7 +1134,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="17" t="s">
-        <x:v>14</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
@@ -1150,13 +1150,13 @@
     </x:row>
     <x:row r="5" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>37</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>32</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>36</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D5" s="21">
         <x:v>15</x:v>
@@ -1165,7 +1165,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="17" t="s">
-        <x:v>1</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5"/>
@@ -1184,10 +1184,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
-        <x:v>20</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C6" s="6" t="s">
-        <x:v>35</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D6" s="21">
         <x:v>20</x:v>
@@ -1196,7 +1196,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="17" t="s">
-        <x:v>2</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5"/>
@@ -1212,13 +1212,13 @@
     </x:row>
     <x:row r="7" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>7</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>31</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D7" s="21">
         <x:v>25</x:v>
@@ -1227,7 +1227,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="F7" s="17" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5"/>
@@ -1243,13 +1243,13 @@
     </x:row>
     <x:row r="8" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A8" s="6" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>23</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
-        <x:v>15</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D8" s="22">
         <x:v>12</x:v>
@@ -1258,7 +1258,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="17" t="s">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5"/>
@@ -1274,13 +1274,13 @@
     </x:row>
     <x:row r="9" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A9" s="7" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>22</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="22">
         <x:v>18</x:v>
@@ -1289,7 +1289,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F9" s="17" t="s">
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="5"/>
@@ -1305,13 +1305,13 @@
     </x:row>
     <x:row r="10" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A10" s="6" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B10" s="6" t="s">
         <x:v>33</x:v>
       </x:c>
       <x:c r="C10" s="6" t="s">
-        <x:v>41</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="21">
         <x:v>24</x:v>
@@ -1320,7 +1320,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="17" t="s">
-        <x:v>0</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G10" s="5"/>
       <x:c r="H10" s="5"/>
@@ -1336,13 +1336,13 @@
     </x:row>
     <x:row r="11" spans="1:17" ht="15.75" customHeight="1">
       <x:c r="A11" s="8" t="s">
-        <x:v>10</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B11" s="8" t="s">
-        <x:v>24</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C11" s="8" t="s">
-        <x:v>17</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D11" s="23">
         <x:v>30</x:v>
@@ -1351,7 +1351,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="17" t="s">
-        <x:v>18</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G11" s="5"/>
       <x:c r="H11" s="5"/>

</xml_diff>

<commit_message>
[Add - Weapon Data] GradeDataId 데이터 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Weapon.xlsx
+++ b/JsonConverter/ExcelFiles/Weapon.xlsx
@@ -19,123 +19,144 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
+  <x:si>
+    <x:t>Grade_Rare</x:t>
+  </x:si>
+  <x:si>
+    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다. (공격력+ 10)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 힘을 이끌어내는 전용 검. (공격력+ 25)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>창술 수련에 사용되는 훈련용 창. (공격력+ 18)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 왕국의 기사단에 지급되는 검. (공격력+ 20)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 검술 훈련에 사용되는 표준 검. (공격력+ 15)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
+  </x:si>
   <x:si>
     <x:t>웰빙리아 왕국 기사단이 사용하는 장창. (공격력+ 24)</x:t>
   </x:si>
   <x:si>
-    <x:t>창술 수련에 사용되는 훈련용 창. (공격력+ 18)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토의 힘을 이끌어내는 전용 검. (공격력+ 25)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 왕국의 기사단에 지급되는 검. (공격력+ 20)</x:t>
+    <x:t>설명</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>이름</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TotoSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토 장창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>나무 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 장창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토의 기사검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
+  </x:si>
+  <x:si>
+    <x:t>요구 레벨</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>훈련용 창</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiredLevel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아 기사검</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다. (공격력+ 30)</x:t>
   </x:si>
   <x:si>
     <x:t>나무를 깎아 만든 간단한 창. 초보 모험가들이 사용한다. (공격력+ 12)</x:t>
   </x:si>
   <x:si>
-    <x:t>토토를 위해 제작된 전용 창. 강력한 힘이 깃들어있다. (공격력+ 30)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TraningSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WoodenSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>이름</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>설명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 검술 훈련에 사용되는 표준 검. (공격력+ 15)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WellbeingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_TrainingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Weapon_WellbeingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RequiredLevel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TotoSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TotoSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>훈련용 검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>훈련용 창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무 검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>나무 창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아 장창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토 장창</x:t>
-  </x:si>
-  <x:si>
-    <x:t>토토의 기사검</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>요구 레벨</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
+    <x:t>GradeDataId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WoodenSpear_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_TrainingSword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_WellbeingSpear_1</x:t>
   </x:si>
   <x:si>
     <x:t>Weapon_TrainingSpear_1</x:t>
@@ -144,19 +165,10 @@
     <x:t>Weapon_WoodenSword_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_WellbeingSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_TrainingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WellbeingSword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_WoodenSpear_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>거칠게 다듬은 나무 검. 초보 모험가들이 사용한다. (공격력+ 10)</x:t>
+    <x:t>Grade_Normal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade_Epic</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -344,7 +356,7 @@
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
@@ -442,6 +454,18 @@
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
@@ -1048,44 +1072,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:Q38"/>
+  <x:dimension ref="A1:R38"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="24.33203125" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="60.4453125" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="12.66796875" style="18" customWidth="1"/>
-    <x:col min="5" max="5" width="14.77734375" style="28" customWidth="1"/>
-    <x:col min="6" max="6" width="43.109375" style="14" customWidth="1"/>
-    <x:col min="7" max="7" width="30.5703125" style="2" customWidth="1"/>
+    <x:col min="5" max="6" width="14.77734375" style="28" customWidth="1"/>
+    <x:col min="7" max="7" width="43.109375" style="14" customWidth="1"/>
+    <x:col min="8" max="8" width="30.5703125" style="2" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:5" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>26</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B1" s="3" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="s">
-        <x:v>14</x:v>
-      </x:c>
       <x:c r="D1" s="19" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="E1" s="29" t="s">
-        <x:v>37</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="F1" s="33"/>
+    </x:row>
+    <x:row r="2" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A2" s="3" t="s">
-        <x:v>38</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D2" s="19" t="s">
         <x:v>13</x:v>
@@ -1093,39 +1118,45 @@
       <x:c r="E2" s="29" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F2" s="15" t="s">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="F2" s="33" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G2" s="15" t="s">
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7" ht="15.75" customHeight="1">
       <x:c r="A3" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B3" s="4" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="C3" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="D3" s="20" t="s">
-        <x:v>31</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E3" s="30" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F3" s="34" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="G3" s="16" t="s">
+        <x:v>38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A4" s="6" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="F3" s="16" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A4" s="6" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="s">
-        <x:v>30</x:v>
-      </x:c>
       <x:c r="C4" s="6" t="s">
-        <x:v>45</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D4" s="21">
         <x:v>10</x:v>
@@ -1133,10 +1164,12 @@
       <x:c r="E4" s="31">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F4" s="17" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G4" s="5"/>
+      <x:c r="F4" s="35" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G4" s="17" t="s">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5"/>
       <x:c r="J4" s="5"/>
@@ -1147,16 +1180,17 @@
       <x:c r="O4" s="5"/>
       <x:c r="P4" s="5"/>
       <x:c r="Q4" s="5"/>
-    </x:row>
-    <x:row r="5" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A5" s="6" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>27</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>15</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D5" s="21">
         <x:v>15</x:v>
@@ -1164,10 +1198,12 @@
       <x:c r="E5" s="31">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F5" s="17" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G5" s="5"/>
+      <x:c r="F5" s="35" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="s">
+        <x:v>34</x:v>
+      </x:c>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5"/>
       <x:c r="J5" s="5"/>
@@ -1178,16 +1214,17 @@
       <x:c r="O5" s="5"/>
       <x:c r="P5" s="5"/>
       <x:c r="Q5" s="5"/>
-    </x:row>
-    <x:row r="6" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
-        <x:v>16</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C6" s="6" t="s">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D6" s="21">
         <x:v>20</x:v>
@@ -1195,10 +1232,12 @@
       <x:c r="E6" s="31">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F6" s="17" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="G6" s="5"/>
+      <x:c r="F6" s="35" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="s">
+        <x:v>33</x:v>
+      </x:c>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5"/>
       <x:c r="J6" s="5"/>
@@ -1209,13 +1248,14 @@
       <x:c r="O6" s="5"/>
       <x:c r="P6" s="5"/>
       <x:c r="Q6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:17" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="R6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:18" s="1" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>23</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>35</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C7" s="6" t="s">
         <x:v>2</x:v>
@@ -1226,10 +1266,12 @@
       <x:c r="E7" s="31">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="F7" s="17" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="G7" s="5"/>
+      <x:c r="F7" s="35" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="s">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
@@ -1240,16 +1282,17 @@
       <x:c r="O7" s="5"/>
       <x:c r="P7" s="5"/>
       <x:c r="Q7" s="5"/>
-    </x:row>
-    <x:row r="8" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A8" s="6" t="s">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B8" s="7" t="s">
-        <x:v>32</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
-        <x:v>4</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D8" s="22">
         <x:v>12</x:v>
@@ -1257,10 +1300,12 @@
       <x:c r="E8" s="31">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F8" s="17" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G8" s="5"/>
+      <x:c r="F8" s="35" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G8" s="17" t="s">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5"/>
       <x:c r="J8" s="5"/>
@@ -1271,16 +1316,17 @@
       <x:c r="O8" s="5"/>
       <x:c r="P8" s="5"/>
       <x:c r="Q8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A9" s="7" t="s">
-        <x:v>39</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B9" s="7" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="22">
         <x:v>18</x:v>
@@ -1288,10 +1334,12 @@
       <x:c r="E9" s="31">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F9" s="17" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G9" s="5"/>
+      <x:c r="F9" s="35" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G9" s="17" t="s">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5"/>
       <x:c r="J9" s="5"/>
@@ -1302,16 +1350,17 @@
       <x:c r="O9" s="5"/>
       <x:c r="P9" s="5"/>
       <x:c r="Q9" s="5"/>
-    </x:row>
-    <x:row r="10" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A10" s="6" t="s">
-        <x:v>41</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B10" s="6" t="s">
-        <x:v>33</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C10" s="6" t="s">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D10" s="21">
         <x:v>24</x:v>
@@ -1319,10 +1368,12 @@
       <x:c r="E10" s="31">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F10" s="17" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="G10" s="5"/>
+      <x:c r="F10" s="35" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="s">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5"/>
       <x:c r="J10" s="5"/>
@@ -1333,16 +1384,17 @@
       <x:c r="O10" s="5"/>
       <x:c r="P10" s="5"/>
       <x:c r="Q10" s="5"/>
-    </x:row>
-    <x:row r="11" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A11" s="8" t="s">
-        <x:v>24</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B11" s="8" t="s">
-        <x:v>34</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" s="8" t="s">
-        <x:v>5</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D11" s="23">
         <x:v>30</x:v>
@@ -1350,10 +1402,12 @@
       <x:c r="E11" s="31">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F11" s="17" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="G11" s="5"/>
+      <x:c r="F11" s="35" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="G11" s="17" t="s">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="H11" s="5"/>
       <x:c r="I11" s="5"/>
       <x:c r="J11" s="5"/>
@@ -1364,15 +1418,16 @@
       <x:c r="O11" s="5"/>
       <x:c r="P11" s="5"/>
       <x:c r="Q11" s="5"/>
-    </x:row>
-    <x:row r="12" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A12" s="8"/>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="8"/>
       <x:c r="D12" s="23"/>
       <x:c r="E12" s="31"/>
-      <x:c r="F12" s="17"/>
-      <x:c r="G12" s="5"/>
+      <x:c r="F12" s="35"/>
+      <x:c r="G12" s="17"/>
       <x:c r="H12" s="5"/>
       <x:c r="I12" s="5"/>
       <x:c r="J12" s="5"/>
@@ -1383,15 +1438,16 @@
       <x:c r="O12" s="5"/>
       <x:c r="P12" s="5"/>
       <x:c r="Q12" s="5"/>
-    </x:row>
-    <x:row r="13" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R12" s="5"/>
+    </x:row>
+    <x:row r="13" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A13" s="9"/>
       <x:c r="B13" s="9"/>
       <x:c r="C13" s="9"/>
       <x:c r="D13" s="24"/>
       <x:c r="E13" s="31"/>
-      <x:c r="F13" s="17"/>
-      <x:c r="G13" s="5"/>
+      <x:c r="F13" s="35"/>
+      <x:c r="G13" s="17"/>
       <x:c r="H13" s="5"/>
       <x:c r="I13" s="5"/>
       <x:c r="J13" s="5"/>
@@ -1402,15 +1458,16 @@
       <x:c r="O13" s="5"/>
       <x:c r="P13" s="5"/>
       <x:c r="Q13" s="5"/>
-    </x:row>
-    <x:row r="14" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R13" s="5"/>
+    </x:row>
+    <x:row r="14" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A14" s="9"/>
       <x:c r="B14" s="9"/>
       <x:c r="C14" s="9"/>
       <x:c r="D14" s="24"/>
       <x:c r="E14" s="31"/>
-      <x:c r="F14" s="17"/>
-      <x:c r="G14" s="5"/>
+      <x:c r="F14" s="35"/>
+      <x:c r="G14" s="17"/>
       <x:c r="H14" s="5"/>
       <x:c r="I14" s="5"/>
       <x:c r="J14" s="5"/>
@@ -1421,15 +1478,16 @@
       <x:c r="O14" s="5"/>
       <x:c r="P14" s="5"/>
       <x:c r="Q14" s="5"/>
-    </x:row>
-    <x:row r="15" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R14" s="5"/>
+    </x:row>
+    <x:row r="15" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A15" s="8"/>
       <x:c r="B15" s="8"/>
       <x:c r="C15" s="8"/>
       <x:c r="D15" s="23"/>
       <x:c r="E15" s="31"/>
-      <x:c r="F15" s="17"/>
-      <x:c r="G15" s="5"/>
+      <x:c r="F15" s="35"/>
+      <x:c r="G15" s="17"/>
       <x:c r="H15" s="5"/>
       <x:c r="I15" s="5"/>
       <x:c r="J15" s="5"/>
@@ -1440,15 +1498,16 @@
       <x:c r="O15" s="5"/>
       <x:c r="P15" s="5"/>
       <x:c r="Q15" s="5"/>
-    </x:row>
-    <x:row r="16" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R15" s="5"/>
+    </x:row>
+    <x:row r="16" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A16" s="6"/>
       <x:c r="B16" s="6"/>
       <x:c r="C16" s="6"/>
       <x:c r="D16" s="21"/>
       <x:c r="E16" s="31"/>
-      <x:c r="F16" s="17"/>
-      <x:c r="G16" s="5"/>
+      <x:c r="F16" s="35"/>
+      <x:c r="G16" s="17"/>
       <x:c r="H16" s="5"/>
       <x:c r="I16" s="5"/>
       <x:c r="J16" s="5"/>
@@ -1459,15 +1518,16 @@
       <x:c r="O16" s="5"/>
       <x:c r="P16" s="5"/>
       <x:c r="Q16" s="5"/>
-    </x:row>
-    <x:row r="17" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R16" s="5"/>
+    </x:row>
+    <x:row r="17" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A17" s="9"/>
       <x:c r="B17" s="9"/>
       <x:c r="C17" s="9"/>
       <x:c r="D17" s="24"/>
       <x:c r="E17" s="31"/>
-      <x:c r="F17" s="17"/>
-      <x:c r="G17" s="5"/>
+      <x:c r="F17" s="35"/>
+      <x:c r="G17" s="17"/>
       <x:c r="H17" s="5"/>
       <x:c r="I17" s="5"/>
       <x:c r="J17" s="5"/>
@@ -1478,15 +1538,16 @@
       <x:c r="O17" s="5"/>
       <x:c r="P17" s="5"/>
       <x:c r="Q17" s="5"/>
-    </x:row>
-    <x:row r="18" spans="1:17" ht="15.75" customHeight="1">
+      <x:c r="R17" s="5"/>
+    </x:row>
+    <x:row r="18" spans="1:18" ht="15.75" customHeight="1">
       <x:c r="A18" s="9"/>
       <x:c r="B18" s="9"/>
       <x:c r="C18" s="9"/>
       <x:c r="D18" s="24"/>
       <x:c r="E18" s="31"/>
-      <x:c r="F18" s="17"/>
-      <x:c r="G18" s="5"/>
+      <x:c r="F18" s="35"/>
+      <x:c r="G18" s="17"/>
       <x:c r="H18" s="5"/>
       <x:c r="I18" s="5"/>
       <x:c r="J18" s="5"/>
@@ -1497,151 +1558,172 @@
       <x:c r="O18" s="5"/>
       <x:c r="P18" s="5"/>
       <x:c r="Q18" s="5"/>
-    </x:row>
-    <x:row r="19" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="R18" s="5"/>
+    </x:row>
+    <x:row r="19" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A19" s="10"/>
       <x:c r="B19" s="10"/>
       <x:c r="C19" s="10"/>
       <x:c r="D19" s="25"/>
       <x:c r="E19" s="32"/>
-    </x:row>
-    <x:row r="20" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F19" s="36"/>
+    </x:row>
+    <x:row r="20" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A20" s="11"/>
       <x:c r="B20" s="11"/>
       <x:c r="C20" s="11"/>
       <x:c r="D20" s="25"/>
       <x:c r="E20" s="32"/>
-    </x:row>
-    <x:row r="21" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F20" s="36"/>
+    </x:row>
+    <x:row r="21" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A21" s="11"/>
       <x:c r="B21" s="11"/>
       <x:c r="C21" s="11"/>
       <x:c r="D21" s="25"/>
       <x:c r="E21" s="32"/>
-    </x:row>
-    <x:row r="22" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F21" s="36"/>
+    </x:row>
+    <x:row r="22" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A22" s="11"/>
       <x:c r="B22" s="11"/>
       <x:c r="C22" s="11"/>
       <x:c r="D22" s="25"/>
       <x:c r="E22" s="32"/>
-      <x:c r="G22" s="5"/>
-    </x:row>
-    <x:row r="23" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F22" s="36"/>
+      <x:c r="H22" s="5"/>
+    </x:row>
+    <x:row r="23" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A23" s="11"/>
       <x:c r="B23" s="11"/>
       <x:c r="C23" s="11"/>
       <x:c r="D23" s="25"/>
       <x:c r="E23" s="32"/>
-    </x:row>
-    <x:row r="24" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F23" s="36"/>
+    </x:row>
+    <x:row r="24" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A24" s="11"/>
       <x:c r="B24" s="11"/>
       <x:c r="C24" s="11"/>
       <x:c r="D24" s="25"/>
       <x:c r="E24" s="32"/>
-    </x:row>
-    <x:row r="25" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F24" s="36"/>
+    </x:row>
+    <x:row r="25" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A25" s="11"/>
       <x:c r="B25" s="11"/>
       <x:c r="C25" s="11"/>
       <x:c r="D25" s="25"/>
       <x:c r="E25" s="32"/>
-    </x:row>
-    <x:row r="26" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F25" s="36"/>
+    </x:row>
+    <x:row r="26" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A26" s="11"/>
       <x:c r="B26" s="11"/>
       <x:c r="C26" s="11"/>
       <x:c r="D26" s="25"/>
       <x:c r="E26" s="32"/>
-    </x:row>
-    <x:row r="27" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F26" s="36"/>
+    </x:row>
+    <x:row r="27" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A27" s="11"/>
       <x:c r="B27" s="11"/>
       <x:c r="C27" s="11"/>
       <x:c r="D27" s="25"/>
       <x:c r="E27" s="32"/>
-    </x:row>
-    <x:row r="28" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F27" s="36"/>
+    </x:row>
+    <x:row r="28" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A28" s="11"/>
       <x:c r="B28" s="11"/>
       <x:c r="C28" s="11"/>
       <x:c r="D28" s="25"/>
       <x:c r="E28" s="32"/>
-      <x:c r="G28" s="5"/>
-    </x:row>
-    <x:row r="29" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F28" s="36"/>
+      <x:c r="H28" s="5"/>
+    </x:row>
+    <x:row r="29" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A29" s="12"/>
       <x:c r="B29" s="12"/>
       <x:c r="C29" s="12"/>
       <x:c r="D29" s="26"/>
       <x:c r="E29" s="32"/>
-      <x:c r="G29" s="5"/>
-    </x:row>
-    <x:row r="30" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F29" s="36"/>
+      <x:c r="H29" s="5"/>
+    </x:row>
+    <x:row r="30" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A30" s="12"/>
       <x:c r="B30" s="12"/>
       <x:c r="C30" s="12"/>
       <x:c r="D30" s="26"/>
       <x:c r="E30" s="32"/>
-      <x:c r="G30" s="5"/>
-    </x:row>
-    <x:row r="31" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="F30" s="36"/>
+      <x:c r="H30" s="5"/>
+    </x:row>
+    <x:row r="31" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A31" s="12"/>
       <x:c r="B31" s="12"/>
       <x:c r="C31" s="12"/>
       <x:c r="D31" s="26"/>
       <x:c r="E31" s="32"/>
-      <x:c r="G31" s="5"/>
-    </x:row>
-    <x:row r="32" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F31" s="36"/>
+      <x:c r="H31" s="5"/>
+    </x:row>
+    <x:row r="32" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A32" s="12"/>
       <x:c r="B32" s="12"/>
       <x:c r="C32" s="12"/>
       <x:c r="D32" s="26"/>
       <x:c r="E32" s="32"/>
-    </x:row>
-    <x:row r="33" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F32" s="36"/>
+    </x:row>
+    <x:row r="33" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A33" s="12"/>
       <x:c r="B33" s="12"/>
       <x:c r="C33" s="12"/>
       <x:c r="D33" s="26"/>
       <x:c r="E33" s="32"/>
-    </x:row>
-    <x:row r="34" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F33" s="36"/>
+    </x:row>
+    <x:row r="34" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A34" s="12"/>
       <x:c r="B34" s="12"/>
       <x:c r="C34" s="12"/>
       <x:c r="D34" s="26"/>
       <x:c r="E34" s="32"/>
-    </x:row>
-    <x:row r="35" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F34" s="36"/>
+    </x:row>
+    <x:row r="35" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A35" s="13"/>
       <x:c r="B35" s="13"/>
       <x:c r="C35" s="13"/>
       <x:c r="D35" s="27"/>
       <x:c r="E35" s="32"/>
-    </x:row>
-    <x:row r="36" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F35" s="36"/>
+    </x:row>
+    <x:row r="36" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A36" s="13"/>
       <x:c r="B36" s="13"/>
       <x:c r="C36" s="13"/>
       <x:c r="D36" s="27"/>
       <x:c r="E36" s="32"/>
-    </x:row>
-    <x:row r="37" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F36" s="36"/>
+    </x:row>
+    <x:row r="37" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A37" s="13"/>
       <x:c r="B37" s="13"/>
       <x:c r="C37" s="13"/>
       <x:c r="D37" s="27"/>
       <x:c r="E37" s="32"/>
-    </x:row>
-    <x:row r="38" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F37" s="36"/>
+    </x:row>
+    <x:row r="38" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A38" s="13"/>
       <x:c r="B38" s="13"/>
       <x:c r="C38" s="13"/>
       <x:c r="D38" s="27"/>
       <x:c r="E38" s="32"/>
+      <x:c r="F38" s="36"/>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1"/>
     <x:row r="40" ht="15.75" customHeight="1"/>

</xml_diff>